<commit_message>
Etkinlik takvimini kesin tarihler ve yeni kongrelerle güncelle
Kongrelerin net tarihleri eklendi (29. TDB, 32. Pedodonti, EDAD 30,
Türk-Yunan Ege Workshop, Endodonti Sempozyumu). Tablo üç bölüme ayrıldı:
ücretsiz/sürekli, yaklaşan kongreler (tarih sırasıyla), 2026'da geçmiş
yıllık etkinlikler.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RpswN2cHxQYsnyjpm4xQAy
</commit_message>
<xml_diff>
--- a/dis_hekimligi_etkinlikler.xlsx
+++ b/dis_hekimligi_etkinlikler.xlsx
@@ -67,7 +67,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -86,12 +86,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="004A7C94"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00E7F4EA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F5F8FA"/>
+        <fgColor rgb="00FBF4E6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F0F0F0"/>
       </patternFill>
     </fill>
   </fills>
@@ -121,7 +131,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -132,41 +142,48 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -533,17 +550,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="52" customWidth="1" min="7" max="7"/>
-    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="50" customWidth="1" min="7" max="7"/>
+    <col width="33" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -556,7 +573,7 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Yeni mezun / genç diş hekimleri için hazırlandı  •  ÜCRETSİZ etkinlikler önce sıralanmıştır  •  Yeşil satırlar = ücretsiz  •  Hazırlık tarihi: 18.08.2026  •  Tarih/ücret bilgileri değişebilir, kayıt öncesi ilgili linki doğrulayın</t>
+          <t>Yeni mezun / genç diş hekimleri için · ÜCRETSİZ ve sürekli etkinlikler önce · kongreler tarih sırasıyla · Hazırlık: 18.08.2026 · Tarih/ücret değişebilir, kayıt öncesi linki doğrulayın</t>
         </is>
       </c>
     </row>
@@ -578,7 +595,7 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Tarih / Sıklık</t>
+          <t>Tarih / Durum</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -602,545 +619,754 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="78" customHeight="1">
-      <c r="A4" s="4" t="n">
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>🟢 ÜCRETSİZ / SÜREKLİ ETKİNLİKLER (yıl boyu — öncelikli)</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n"/>
+      <c r="C4" s="5" t="n"/>
+      <c r="D4" s="5" t="n"/>
+      <c r="E4" s="5" t="n"/>
+      <c r="F4" s="5" t="n"/>
+      <c r="G4" s="5" t="n"/>
+      <c r="H4" s="5" t="n"/>
+    </row>
+    <row r="5" ht="80" customHeight="1">
+      <c r="A5" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>TDB Akademi Online Bilimsel Etkinlikleri</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>Türk Dişhekimleri Birliği (TDB) Akademi</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>Yıl boyu düzenli (Zoom + YouTube)</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Yıl boyu düzenli · Zoom + TDB YouTube · kayıt zorunlu</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
         <is>
           <t>Online</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr">
+      <c r="F5" s="8" t="inlineStr">
         <is>
           <t>Ücretsiz</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
-        <is>
-          <t>Mezuniyet sonrası sürekli eğitimin en güvenilir ücretsiz kaynağı. Güncel klinik konular, alanında uzman hocalarla. Kayıt zorunlu, tüm meslektaşlara açık. Yeni mezun bir hekim için ideal başlangıç.</t>
-        </is>
-      </c>
-      <c r="H4" s="7" t="inlineStr">
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>Mezuniyet sonrası sürekli eğitimin en güvenilir ücretsiz kaynağı. Güncel klinik konular, alanında uzman hocalarla. Yeni mezun bir hekim için ideal başlangıç.</t>
+        </is>
+      </c>
+      <c r="H5" s="9" t="inlineStr">
         <is>
           <t>https://tdbakademi.org</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="78" customHeight="1">
-      <c r="A5" s="4" t="n">
+    <row r="6" ht="80" customHeight="1">
+      <c r="A6" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>VESTALKS Canlı Webinar Serisi</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>Dr. Vesta (Diş Hekimliği Eğitim Platformu)</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>Her Salı 20:00 (canlı)</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>Her Salı 20:00 (canlı) · yıl boyu</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
         <is>
           <t>Online</t>
         </is>
       </c>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="F6" s="8" t="inlineStr">
         <is>
           <t>Ücretsiz</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>Üyelik ve canlı yayınlar tamamen ücretsiz. Klinik yaklaşımlar, mesleki yenilikler ve kariyer (yurtdışı/İngiltere) içerikleri. Denizli'den evden katılıma çok uygun.</t>
-        </is>
-      </c>
-      <c r="H5" s="7" t="inlineStr">
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>Üyelik ve canlı yayınlar tamamen ücretsiz. Klinik yaklaşımlar, mesleki yenilikler ve yurtdışı (İngiltere) kariyer içerikleri. Denizli'den evden katılıma çok uygun.</t>
+        </is>
+      </c>
+      <c r="H6" s="9" t="inlineStr">
         <is>
           <t>https://www.drvesta.com</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="78" customHeight="1">
-      <c r="A6" s="4" t="n">
+    <row r="7" ht="80" customHeight="1">
+      <c r="A7" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>Dentsply Sirona Academy – Web Seminerleri</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>Dentsply Sirona (firma akademisi)</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>Yıl boyu (takvimli)</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>Yıl boyu · takvimli web seminerleri + kayıtlı videolar</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
         <is>
           <t>Online + bazıları Yüz Yüze</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="F7" s="8" t="inlineStr">
         <is>
           <t>Ücretsiz</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>Web seminerleri, kendi hızında online eğitim ve eğitim videolarının çoğu ücretsiz. Endodonti, restoratif ve dijital diş hekimliği ekipman/teknik odaklı pratik içerik.</t>
-        </is>
-      </c>
-      <c r="H6" s="7" t="inlineStr">
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>Web seminerleri, kendi hızında online eğitim ve videoların çoğu ücretsiz. Endodonti, restoratif ve dijital diş hekimliği odaklı pratik içerik.</t>
+        </is>
+      </c>
+      <c r="H7" s="9" t="inlineStr">
         <is>
           <t>https://www.dentsplysirona.com/tr-tr/akademi/surekli-egitim.html</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="78" customHeight="1">
-      <c r="A7" s="4" t="n">
+    <row r="8" ht="80" customHeight="1">
+      <c r="A8" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>İzmir Dişhekimleri Odası (İZDO) Meslek İçi Eğitimler</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C8" s="7" t="inlineStr">
         <is>
           <t>İzmir Dişhekimleri Odası</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>Yıl boyu (duyurulara göre)</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>Yıl boyu · duyurulara göre</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
         <is>
           <t>İzmir – Yüz Yüze / bazıları Online</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr">
+      <c r="F8" s="8" t="inlineStr">
         <is>
           <t>Ücretsiz</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="G8" s="7" t="inlineStr">
         <is>
           <t>Oda üyelerine yönelik seminer ve kurslar genelde ücretsiz. İzmir, Denizli'ye en yakın büyük eğitim merkezi; yüz yüze networking fırsatı.</t>
         </is>
       </c>
-      <c r="H7" s="7" t="inlineStr">
+      <c r="H8" s="9" t="inlineStr">
         <is>
           <t>https://izdo.org/Duyuru</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="78" customHeight="1">
-      <c r="A8" s="4" t="n">
+    <row r="9" ht="80" customHeight="1">
+      <c r="A9" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>Denizli Dişhekimleri Odası Bilimsel Etkinlikleri</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>Denizli Dişhekimleri Odası</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Yıl boyu (duyurulara göre)</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>Yıl boyu · duyurulara göre</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
         <is>
           <t>Denizli – Yüz Yüze</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr">
+      <c r="F9" s="8" t="inlineStr">
         <is>
           <t>Ücretsiz</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
-        <is>
-          <t>Kendi şehrinizde, üyelere ücretsiz/indirimli klinik odaklı seminerler. Yerel meslektaşlarla tanışmak ve oda etkinliklerini takip etmek için birincil kaynak.</t>
-        </is>
-      </c>
-      <c r="H8" s="7" t="inlineStr">
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>Kendi şehrinizde, üyelere ücretsiz/indirimli klinik odaklı seminerler. Yerel meslektaşlarla tanışmak için birincil kaynak; oda kaydınız üzerinden takip edin.</t>
+        </is>
+      </c>
+      <c r="H9" s="9" t="inlineStr">
         <is>
           <t>https://denizli-dho.org.tr</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="78" customHeight="1">
-      <c r="A9" s="4" t="n">
+    <row r="10" ht="80" customHeight="1">
+      <c r="A10" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>İstanbul Dişhekimleri Odası (İDO) Sürekli Eğitim</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C10" s="7" t="inlineStr">
         <is>
           <t>İstanbul Dişhekimleri Odası</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>Yıl boyu (duyurulara göre)</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>Yıl boyu · duyurulara göre</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
         <is>
           <t>İstanbul – Yüz Yüze / Online</t>
         </is>
       </c>
-      <c r="F9" s="6" t="inlineStr">
+      <c r="F10" s="8" t="inlineStr">
         <is>
           <t>Ücretsiz</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr">
-        <is>
-          <t>Türkiye'nin en büyük odası; üyelere yönelik zengin ve çoğu ücretsiz meslek içi eğitim programı. Online yayınları Denizli'den de izlenebilir.</t>
-        </is>
-      </c>
-      <c r="H9" s="7" t="inlineStr">
-        <is>
-          <t>https://www.ido.org.tr</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="78" customHeight="1">
-      <c r="A10" s="4" t="n">
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>Türkiye'nin en büyük odası; üyelere yönelik zengin ve çoğu ücretsiz meslek içi eğitim. Online yayınları Denizli'den de izlenebilir.</t>
+        </is>
+      </c>
+      <c r="H10" s="9" t="inlineStr">
+        <is>
+          <t>https://www.ido.org.tr/etkinlikler/</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="80" customHeight="1">
+      <c r="A11" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>Genç Diş Hekimliği Derneği (GDHDER) Etkinlikleri</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>Genç Diş Hekimliği Derneği</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>Yıl boyu (webinar + buluşma)</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>Yıl boyu · webinar + buluşma</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
         <is>
           <t>Online + Yüz Yüze</t>
         </is>
       </c>
-      <c r="F10" s="6" t="inlineStr">
+      <c r="F11" s="8" t="inlineStr">
         <is>
           <t>Ücretsiz</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr">
-        <is>
-          <t>Tam da sizin profilinize (yeni mezun, 25 yaş) yönelik dernek. Kariyer, girişim ve klinik başlangıç webinarları; genç hekim topluluğu ve mentorluk.</t>
-        </is>
-      </c>
-      <c r="H10" s="7" t="inlineStr">
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>Tam profilinize (yeni mezun, 25 yaş) yönelik dernek. Kariyer, girişim ve klinik başlangıç webinarları; genç hekim topluluğu ve mentorluk.</t>
+        </is>
+      </c>
+      <c r="H11" s="9" t="inlineStr">
         <is>
           <t>https://gdhder.org.tr</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="78" customHeight="1">
-      <c r="A11" s="4" t="n">
+    <row r="12" ht="80" customHeight="1">
+      <c r="A12" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>Nobel Biocare / Firma İmplant Webinarları (YouTube)</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Nobel Biocare / Firma İmplant Webinarları</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
         <is>
           <t>Nobel Biocare Türkiye vb. firma akademileri</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>Düzenli / arşiv</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>Düzenli canlı + arşiv (YouTube)</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
         <is>
           <t>Online</t>
         </is>
       </c>
-      <c r="F11" s="6" t="inlineStr">
+      <c r="F12" s="8" t="inlineStr">
         <is>
           <t>Ücretsiz</t>
         </is>
       </c>
-      <c r="G11" s="5" t="inlineStr">
-        <is>
-          <t>İmplantoloji ve dijital iş akışına giriş için ücretsiz canlı ve kayıtlı webinarlar. Yeni mezun için implant konusunda temel oluşturur.</t>
-        </is>
-      </c>
-      <c r="H11" s="7" t="inlineStr">
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>İmplantoloji ve dijital iş akışına giriş için ücretsiz canlı ve kayıtlı webinarlar. Yeni mezun için implant konusunda sağlam temel.</t>
+        </is>
+      </c>
+      <c r="H12" s="9" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@nobelbiocareturkiye</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="78" customHeight="1">
-      <c r="A12" s="4" t="n">
+    <row r="13" ht="80" customHeight="1">
+      <c r="A13" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>Dentiss.com Etkinlik &amp; Webinar Duyuruları</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="C13" s="7" t="inlineStr">
         <is>
           <t>Dentiss (dental portal)</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>Güncel liste</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>Online + Yüz Yüze (aggregator)</t>
-        </is>
-      </c>
-      <c r="F12" s="6" t="inlineStr">
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>Güncel liste · sürekli güncellenir</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>Online + Yüz Yüze (toplu liste)</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
         <is>
           <t>Ücretsiz</t>
         </is>
       </c>
-      <c r="G12" s="5" t="inlineStr">
-        <is>
-          <t>Türkiye'deki webinar, kongre ve fuarları tek yerden takip etmenizi sağlayan ücretsiz portal. Kaçırmamak için düzenli kontrol edin.</t>
-        </is>
-      </c>
-      <c r="H12" s="7" t="inlineStr">
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>Türkiye'deki webinar, kongre ve fuarları tek yerden takip etmenizi sağlar. Yeni etkinlikleri kaçırmamak için düzenli kontrol edin.</t>
+        </is>
+      </c>
+      <c r="H13" s="9" t="inlineStr">
         <is>
           <t>https://www.dentiss.com/kongre-fuar-a16-b50.html</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="78" customHeight="1">
-      <c r="A13" s="4" t="n">
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>🟡 YAKLAŞAN KONGRE &amp; SEMPOZYUMLAR (2026 — tarih sırasıyla)</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n"/>
+      <c r="C14" s="5" t="n"/>
+      <c r="D14" s="5" t="n"/>
+      <c r="E14" s="5" t="n"/>
+      <c r="F14" s="5" t="n"/>
+      <c r="G14" s="5" t="n"/>
+      <c r="H14" s="5" t="n"/>
+    </row>
+    <row r="15" ht="80" customHeight="1">
+      <c r="A15" s="10" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>IDEX İstanbul – Uluslararası Dental Fuar (fuar girişi)</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>29. TDB Uluslararası Dişhekimliği Kongresi</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="inlineStr">
+        <is>
+          <t>Türk Dişhekimleri Birliği (TDB 40. yıl)</t>
+        </is>
+      </c>
+      <c r="D15" s="11" t="inlineStr">
+        <is>
+          <t>1–4 Ekim 2026 · İstanbul Kongre Merkezi · YAKLAŞAN</t>
+        </is>
+      </c>
+      <c r="E15" s="11" t="inlineStr">
+        <is>
+          <t>İstanbul – Yüz Yüze</t>
+        </is>
+      </c>
+      <c r="F15" s="12" t="inlineStr">
+        <is>
+          <t>Ücretli</t>
+        </is>
+      </c>
+      <c r="G15" s="11" t="inlineStr">
+        <is>
+          <t>Türkiye'nin en büyük dişhekimliği kongresi. Öğrenci/genç hekim ve erken kayıt indirimleri, ilk 500 kişiye özel fırsat. Kapsamlı bilimsel program, kurs ve paneller.</t>
+        </is>
+      </c>
+      <c r="H15" s="13" t="inlineStr">
+        <is>
+          <t>https://www.tdbkongreleri.org</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="80" customHeight="1">
+      <c r="A16" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>32. Uluslararası Türk Pedodonti Derneği Kongresi</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>Türk Pedodonti Derneği</t>
+        </is>
+      </c>
+      <c r="D16" s="11" t="inlineStr">
+        <is>
+          <t>10–13 Ekim 2026 · Susesi Luxury Resort, Antalya · YAKLAŞAN</t>
+        </is>
+      </c>
+      <c r="E16" s="11" t="inlineStr">
+        <is>
+          <t>Antalya – Yüz Yüze</t>
+        </is>
+      </c>
+      <c r="F16" s="12" t="inlineStr">
+        <is>
+          <t>Ücretli</t>
+        </is>
+      </c>
+      <c r="G16" s="11" t="inlineStr">
+        <is>
+          <t>Çocuk diş hekimliğine ilgi duyuyorsanız alanın en kapsamlı kongresi. Uygulamalı workshop'lar; genel pratikte pediatrik hasta yönetimi için değerli.</t>
+        </is>
+      </c>
+      <c r="H16" s="13" t="inlineStr">
+        <is>
+          <t>https://www.turkpedo2026.org</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="80" customHeight="1">
+      <c r="A17" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>Ege'nin İki Yakası – Türk-Yunan ILD&amp;PH Workshop 3</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="inlineStr">
+        <is>
+          <t>Ege Üniversitesi Diş Hekimliği Fakültesi</t>
+        </is>
+      </c>
+      <c r="D17" s="11" t="inlineStr">
+        <is>
+          <t>29 Ekim–1 Kasım 2026 · Ege Üniv. Diş Hek. Fak., İzmir · YAKLAŞAN</t>
+        </is>
+      </c>
+      <c r="E17" s="11" t="inlineStr">
+        <is>
+          <t>İzmir – Yüz Yüze</t>
+        </is>
+      </c>
+      <c r="F17" s="12" t="inlineStr">
+        <is>
+          <t>Ücretli</t>
+        </is>
+      </c>
+      <c r="G17" s="11" t="inlineStr">
+        <is>
+          <t>Denizli'ye yakın, uluslararası (Türk-Yunan) uygulamalı workshop. Akademik ortamda periodontoloji/oral tıp odaklı pratik eğitim ve networking.</t>
+        </is>
+      </c>
+      <c r="H17" s="13" t="inlineStr">
+        <is>
+          <t>https://dent.ege.edu.tr</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="80" customHeight="1">
+      <c r="A18" s="10" t="n">
+        <v>13</v>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>30. Uluslararası Estetik Diş Hekimliği Kongresi (EDAD)</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>Estetik Diş Hekimliği Derneği (EDAD)</t>
+        </is>
+      </c>
+      <c r="D18" s="11" t="inlineStr">
+        <is>
+          <t>12–14 Kasım 2026 · Swissôtel The Bosphorus, İstanbul · YAKLAŞAN</t>
+        </is>
+      </c>
+      <c r="E18" s="11" t="inlineStr">
+        <is>
+          <t>İstanbul – Yüz Yüze</t>
+        </is>
+      </c>
+      <c r="F18" s="12" t="inlineStr">
+        <is>
+          <t>Ücretli</t>
+        </is>
+      </c>
+      <c r="G18" s="11" t="inlineStr">
+        <is>
+          <t>'Estetikte 30 Yıl' temalı kongre. Estetik/restoratif ve dijital gülüş tasarımına ilgi duyan genç hekim için birebir; workshop ve geniş sergi alanı.</t>
+        </is>
+      </c>
+      <c r="H18" s="13" t="inlineStr">
+        <is>
+          <t>https://edad2026.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="80" customHeight="1">
+      <c r="A19" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>33. İZDO Uluslararası Bilimsel Kongre ve Sergisi</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="inlineStr">
+        <is>
+          <t>İzmir Dişhekimleri Odası</t>
+        </is>
+      </c>
+      <c r="D19" s="11" t="inlineStr">
+        <is>
+          <t>Kasım 2026 (tahmini – tarih henüz netleşmedi) · İzmir</t>
+        </is>
+      </c>
+      <c r="E19" s="11" t="inlineStr">
+        <is>
+          <t>İzmir – Yüz Yüze</t>
+        </is>
+      </c>
+      <c r="F19" s="12" t="inlineStr">
+        <is>
+          <t>Ücretli</t>
+        </is>
+      </c>
+      <c r="G19" s="11" t="inlineStr">
+        <is>
+          <t>Denizli'ye en yakın büyük uluslararası kongre. Konferans, seminer, kurs + sergi. Genç hekim indirimlerini ve kesin tarihi izdo.org'dan takip edin.</t>
+        </is>
+      </c>
+      <c r="H19" s="13" t="inlineStr">
+        <is>
+          <t>https://www.izdokongreleri.org</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>⚪ 2026'DA GEÇTİ – YILLIK / SONRAKİ EDİSYON İÇİN TAKİP EDİN</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n"/>
+      <c r="C20" s="5" t="n"/>
+      <c r="D20" s="5" t="n"/>
+      <c r="E20" s="5" t="n"/>
+      <c r="F20" s="5" t="n"/>
+      <c r="G20" s="5" t="n"/>
+      <c r="H20" s="5" t="n"/>
+    </row>
+    <row r="21" ht="80" customHeight="1">
+      <c r="A21" s="14" t="n">
+        <v>15</v>
+      </c>
+      <c r="B21" s="15" t="inlineStr">
+        <is>
+          <t>EBDO – Ege Bölgesi Dişhekimleri Odaları Kongresi</t>
+        </is>
+      </c>
+      <c r="C21" s="15" t="inlineStr">
+        <is>
+          <t>Ege Bölgesi Odaları (İZDO öncülüğünde)</t>
+        </is>
+      </c>
+      <c r="D21" s="15" t="inlineStr">
+        <is>
+          <t>27–29 Mart 2026 yapıldı · Pamukkale Kongre Merkezi, Denizli · sonraki edisyon</t>
+        </is>
+      </c>
+      <c r="E21" s="15" t="inlineStr">
+        <is>
+          <t>Denizli/Ege – Yüz Yüze</t>
+        </is>
+      </c>
+      <c r="F21" s="16" t="inlineStr">
+        <is>
+          <t>Ücretli</t>
+        </is>
+      </c>
+      <c r="G21" s="15" t="inlineStr">
+        <is>
+          <t>Bölgesel kongre; 2. edisyonu tam Denizli'de yapıldı. Uygulamalı eğitim + güçlü yerel networking. Bir sonraki edisyon için oda duyurularını izleyin.</t>
+        </is>
+      </c>
+      <c r="H21" s="17" t="inlineStr">
+        <is>
+          <t>https://izdo.org/Duyuru</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="80" customHeight="1">
+      <c r="A22" s="14" t="n">
+        <v>16</v>
+      </c>
+      <c r="B22" s="15" t="inlineStr">
+        <is>
+          <t>IDEX İstanbul – Uluslararası Dental Fuar</t>
+        </is>
+      </c>
+      <c r="C22" s="15" t="inlineStr">
         <is>
           <t>IDEX / TDB işbirliği</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>Yıllık – İstanbul (genelde Nisan)</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
+      <c r="D22" s="15" t="inlineStr">
+        <is>
+          <t>15–18 Nisan 2026 yapıldı · yıllık · fuar girişi genelde ÜCRETSİZ</t>
+        </is>
+      </c>
+      <c r="E22" s="15" t="inlineStr">
         <is>
           <t>İstanbul – Yüz Yüze</t>
         </is>
       </c>
-      <c r="F13" s="6" t="inlineStr">
+      <c r="F22" s="18" t="inlineStr">
         <is>
           <t>Ücretsiz</t>
         </is>
       </c>
-      <c r="G13" s="5" t="inlineStr">
-        <is>
-          <t>Fuar alanına ön kayıtla giriş genelde ÜCRETSİZ. En yeni ürün/teknolojiler, firma standları ve ücretsiz workshop'lar. Bir sonraki edisyonu için kayıt olun.</t>
-        </is>
-      </c>
-      <c r="H13" s="7" t="inlineStr">
+      <c r="G22" s="15" t="inlineStr">
+        <is>
+          <t>Fuar alanına ön kayıtla giriş genelde ücretsiz. En yeni ürün/teknolojiler, firma standları, ücretsiz workshop'lar. Bir sonraki edisyona kaydolun.</t>
+        </is>
+      </c>
+      <c r="H22" s="17" t="inlineStr">
         <is>
           <t>https://www.idex.org.tr</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="78" customHeight="1">
-      <c r="A14" s="8" t="n">
-        <v>11</v>
-      </c>
-      <c r="B14" s="9" t="inlineStr">
-        <is>
-          <t>29. TDB Uluslararası Dişhekimliği Kongresi</t>
-        </is>
-      </c>
-      <c r="C14" s="9" t="inlineStr">
-        <is>
-          <t>Türk Dişhekimleri Birliği</t>
-        </is>
-      </c>
-      <c r="D14" s="9" t="inlineStr">
-        <is>
-          <t>1–4 Ekim 2026 – İstanbul Kongre Merkezi</t>
-        </is>
-      </c>
-      <c r="E14" s="9" t="inlineStr">
-        <is>
-          <t>İstanbul – Yüz Yüze</t>
-        </is>
-      </c>
-      <c r="F14" s="10" t="inlineStr">
+    <row r="23" ht="80" customHeight="1">
+      <c r="A23" s="14" t="n">
+        <v>17</v>
+      </c>
+      <c r="B23" s="15" t="inlineStr">
+        <is>
+          <t>11. Uluslararası Endodonti Sempozyumu</t>
+        </is>
+      </c>
+      <c r="C23" s="15" t="inlineStr">
+        <is>
+          <t>Türk Endodonti Derneği</t>
+        </is>
+      </c>
+      <c r="D23" s="15" t="inlineStr">
+        <is>
+          <t>18–21 Mayıs 2026 yapıldı · Grand Mercure, Ankara · sonraki edisyon</t>
+        </is>
+      </c>
+      <c r="E23" s="15" t="inlineStr">
+        <is>
+          <t>Ankara – Yüz Yüze</t>
+        </is>
+      </c>
+      <c r="F23" s="16" t="inlineStr">
         <is>
           <t>Ücretli</t>
         </is>
       </c>
-      <c r="G14" s="9" t="inlineStr">
-        <is>
-          <t>Türkiye'nin en büyük dişhekimliği kongresi; TDB'nin 40. yılı. Öğrenci/genç hekim ve erken kayıt indirimleri var. Kapsamlı bilimsel program, kurs ve paneller.</t>
-        </is>
-      </c>
-      <c r="H14" s="11" t="inlineStr">
-        <is>
-          <t>https://www.tdbkongreleri.org</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="78" customHeight="1">
-      <c r="A15" s="12" t="n">
-        <v>12</v>
-      </c>
-      <c r="B15" s="13" t="inlineStr">
-        <is>
-          <t>33. İZDO Uluslararası Bilimsel Kongre ve Sergisi</t>
-        </is>
-      </c>
-      <c r="C15" s="13" t="inlineStr">
-        <is>
-          <t>İzmir Dişhekimleri Odası</t>
-        </is>
-      </c>
-      <c r="D15" s="13" t="inlineStr">
-        <is>
-          <t>Kasım 2026 (tahmini) – İzmir</t>
-        </is>
-      </c>
-      <c r="E15" s="13" t="inlineStr">
-        <is>
-          <t>İzmir – Yüz Yüze</t>
-        </is>
-      </c>
-      <c r="F15" s="14" t="inlineStr">
-        <is>
-          <t>Ücretli</t>
-        </is>
-      </c>
-      <c r="G15" s="13" t="inlineStr">
-        <is>
-          <t>Denizli'ye en yakın büyük uluslararası kongre. Konferans, seminer ve kurslarla güncel bilgi + sergi alanı. Genç hekim indirimlerini takip edin.</t>
-        </is>
-      </c>
-      <c r="H15" s="15" t="inlineStr">
-        <is>
-          <t>https://www.izdokongreleri.org</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="78" customHeight="1">
-      <c r="A16" s="8" t="n">
-        <v>13</v>
-      </c>
-      <c r="B16" s="9" t="inlineStr">
-        <is>
-          <t>Ege Bölgesi Dişhekimleri Odaları (EBDO) Kongresi</t>
-        </is>
-      </c>
-      <c r="C16" s="9" t="inlineStr">
-        <is>
-          <t>Ege Bölgesi Odaları (İZDO öncülüğünde)</t>
-        </is>
-      </c>
-      <c r="D16" s="9" t="inlineStr">
-        <is>
-          <t>Yıllık (2026 Denizli'de yapıldı; sonraki edisyon)</t>
-        </is>
-      </c>
-      <c r="E16" s="9" t="inlineStr">
-        <is>
-          <t>Ege bölgesi – Yüz Yüze</t>
-        </is>
-      </c>
-      <c r="F16" s="10" t="inlineStr">
-        <is>
-          <t>Ücretli</t>
-        </is>
-      </c>
-      <c r="G16" s="9" t="inlineStr">
-        <is>
-          <t>Bölgesel kongre; 2. edisyonu Denizli Pamukkale Kongre Merkezi'nde yapıldı. Uygulamalı eğitimler ve bölge hekimleriyle güçlü networking.</t>
-        </is>
-      </c>
-      <c r="H16" s="11" t="inlineStr">
-        <is>
-          <t>https://izdo.org/Duyuru</t>
+      <c r="G23" s="15" t="inlineStr">
+        <is>
+          <t>Kanal tedavisi (endodonti) alanının en güncel sempozyumu. Genel pratikte en sık yapılan işlemlerden biri; sonraki edisyonu takibe değer.</t>
+        </is>
+      </c>
+      <c r="H23" s="17" t="inlineStr">
+        <is>
+          <t>https://endodonti2026.org</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="5">
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A20:H20"/>
     <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A14:H14"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId17"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>